<commit_message>
corrected active commuting algorithm
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements-NHATS.xlsx
+++ b/longitudinal/data_processing_elements-NHATS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17bc974f5891b333/Documents/ProPASS/Harmo/NHATS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="258" documentId="8_{5005C4B8-8269-4712-9267-05709C8265AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FED70469-1339-404C-8A98-A1EF8C446BEC}"/>
+  <xr:revisionPtr revIDLastSave="259" documentId="8_{5005C4B8-8269-4712-9267-05709C8265AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{339FDDB2-46A3-461B-A141-A096D22A068A}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F744FAC3-0BAB-4C7A-92B3-0824573F48DB}"/>
   </bookViews>
@@ -1472,13 +1472,6 @@
   </si>
   <si>
     <t>case_when(
-dt11getoplcs1 == 1 | ha11howgtstr7 == 1 ~ 1;
-dt11getoplcs1 == 2 &amp; ha11howgtstr7 == 2 ~ 0;
-TRUE ~ NA_integer_
-)</t>
-  </si>
-  <si>
-    <t>case_when(
   hw12howtallft %in% c(-7, -8, -9, -1) |
     hw12howtallin %in% c(-7, -8, -9, -1) |
     hw12currweigh %in% c(-7, -8, -9, -1) ~ NA_real_,
@@ -1636,6 +1629,13 @@
 1 = YES;
 2 = NO
 7 = PREVIOUSLY REPORTED</t>
+  </si>
+  <si>
+    <t>case_when(
+dt12getoplcs1 == 1 | ha12howgtstr7 == 1 ~ 1;
+dt12getoplcs1 == 2 &amp; ha12howgtstr7 == 2 ~ 0;
+TRUE ~ NA_integer_
+)</t>
   </si>
 </sst>
 </file>
@@ -2399,7 +2399,7 @@
         <v>14</v>
       </c>
       <c r="Y4" s="11" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="5" spans="1:25" ht="85.5" x14ac:dyDescent="0.45">
@@ -2428,10 +2428,10 @@
         <v>378</v>
       </c>
       <c r="J5" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="K5" t="s">
         <v>401</v>
-      </c>
-      <c r="K5" t="s">
-        <v>402</v>
       </c>
       <c r="L5" s="5" t="s">
         <v>286</v>
@@ -2994,13 +2994,13 @@
         <v>378</v>
       </c>
       <c r="J15" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>373</v>
       </c>
       <c r="L15" s="5" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="N15" t="s">
         <v>315</v>
@@ -3025,7 +3025,7 @@
         <v>14</v>
       </c>
       <c r="Y15" s="11" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="16" spans="1:25" ht="128.25" x14ac:dyDescent="0.45">
@@ -3303,7 +3303,7 @@
         <v>51</v>
       </c>
       <c r="X20" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="21" spans="1:24" ht="15.75" x14ac:dyDescent="0.45">
@@ -4632,10 +4632,10 @@
         <v>38</v>
       </c>
       <c r="X48" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="Y48" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="49" spans="1:25" ht="213.75" x14ac:dyDescent="0.45">
@@ -5483,7 +5483,7 @@
         <v>355</v>
       </c>
       <c r="L66" s="5" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M66" s="5"/>
       <c r="N66" t="s">
@@ -5507,7 +5507,7 @@
         <v>38</v>
       </c>
       <c r="X66" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="Y66" s="2"/>
     </row>
@@ -6137,10 +6137,10 @@
         <v>378</v>
       </c>
       <c r="J80" t="s">
+        <v>389</v>
+      </c>
+      <c r="K80" t="s">
         <v>390</v>
-      </c>
-      <c r="K80" t="s">
-        <v>391</v>
       </c>
       <c r="L80" s="5" t="s">
         <v>310</v>
@@ -6167,10 +6167,10 @@
         <v>51</v>
       </c>
       <c r="X80" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="Y80" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="81" spans="1:25" ht="99.75" x14ac:dyDescent="0.45">
@@ -6228,7 +6228,7 @@
         <v>51</v>
       </c>
       <c r="X81" s="2" t="s">
-        <v>384</v>
+        <v>404</v>
       </c>
     </row>
     <row r="82" spans="1:25" ht="409.5" x14ac:dyDescent="0.45">
@@ -6257,13 +6257,13 @@
         <v>378</v>
       </c>
       <c r="J82" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="K82" s="2" t="s">
         <v>394</v>
       </c>
-      <c r="K82" s="2" t="s">
+      <c r="L82" s="5" t="s">
         <v>395</v>
-      </c>
-      <c r="L82" s="5" t="s">
-        <v>396</v>
       </c>
       <c r="M82" s="5"/>
       <c r="N82" t="s">
@@ -6287,10 +6287,10 @@
         <v>38</v>
       </c>
       <c r="X82" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="Y82" s="2" t="s">
         <v>397</v>
-      </c>
-      <c r="Y82" s="2" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="83" spans="1:25" ht="28.5" x14ac:dyDescent="0.45">

</xml_diff>